<commit_message>
score: refresh OpenLA500 reference
</commit_message>
<xml_diff>
--- a/final_score.xlsx
+++ b/final_score.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="68">
   <si>
     <t xml:space="preserve">队名</t>
   </si>
@@ -301,121 +301,61 @@
     <t xml:space="preserve">0</t>
   </si>
   <si>
-    <t xml:space="preserve">00053E26</t>
-  </si>
-  <si>
     <t xml:space="preserve">bubble_sort</t>
   </si>
   <si>
-    <t xml:space="preserve">00186560</t>
-  </si>
-  <si>
     <t xml:space="preserve">coremark</t>
   </si>
   <si>
-    <t xml:space="preserve">003F1F59</t>
-  </si>
-  <si>
     <t xml:space="preserve">crc32</t>
   </si>
   <si>
-    <t xml:space="preserve">002769F9</t>
-  </si>
-  <si>
     <t xml:space="preserve">dhrystone</t>
   </si>
   <si>
-    <t xml:space="preserve">0000B7A6</t>
-  </si>
-  <si>
     <t xml:space="preserve">quick_sort</t>
   </si>
   <si>
-    <t xml:space="preserve">001E0680</t>
-  </si>
-  <si>
     <t xml:space="preserve">select_sort</t>
   </si>
   <si>
-    <t xml:space="preserve">000FE287</t>
-  </si>
-  <si>
     <t xml:space="preserve">sha</t>
   </si>
   <si>
-    <t xml:space="preserve">00215BBA</t>
-  </si>
-  <si>
     <t xml:space="preserve">stream_copy</t>
   </si>
   <si>
-    <t xml:space="preserve">0001FC67</t>
-  </si>
-  <si>
     <t xml:space="preserve">stringsearch</t>
   </si>
   <si>
-    <t xml:space="preserve">0008E077</t>
-  </si>
-  <si>
     <t xml:space="preserve">fireye_A0</t>
   </si>
   <si>
-    <t xml:space="preserve">0040B822</t>
-  </si>
-  <si>
     <t xml:space="preserve">fireye_B2</t>
   </si>
   <si>
-    <t xml:space="preserve">00084622</t>
-  </si>
-  <si>
     <t xml:space="preserve">fireye_C0</t>
   </si>
   <si>
-    <t xml:space="preserve">000A51E9</t>
-  </si>
-  <si>
     <t xml:space="preserve">fireye_D1</t>
   </si>
   <si>
-    <t xml:space="preserve">005BC44F</t>
-  </si>
-  <si>
     <t xml:space="preserve">fireye_I2</t>
   </si>
   <si>
-    <t xml:space="preserve">003BA045</t>
-  </si>
-  <si>
     <t xml:space="preserve">inner_product</t>
   </si>
   <si>
-    <t xml:space="preserve">00F7A093</t>
-  </si>
-  <si>
     <t xml:space="preserve">lookup_table</t>
   </si>
   <si>
-    <t xml:space="preserve">002D131A</t>
-  </si>
-  <si>
     <t xml:space="preserve">loop_induction</t>
   </si>
   <si>
-    <t xml:space="preserve">00A913D8</t>
-  </si>
-  <si>
     <t xml:space="preserve">my_memcmp</t>
   </si>
   <si>
-    <t xml:space="preserve">0033EE87</t>
-  </si>
-  <si>
     <t xml:space="preserve">minmax_sequence</t>
-  </si>
-  <si>
-    <t xml:space="preserve">003C2869</t>
   </si>
   <si>
     <t xml:space="preserve">三、系统测试分数计算</t>
@@ -635,66 +575,6 @@
   </si>
   <si>
     <t xml:space="preserve">数码管显示(SoC count)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">00100A2E</t>
-  </si>
-  <si>
-    <t xml:space="preserve">004A9290</t>
-  </si>
-  <si>
-    <t xml:space="preserve">00C0ECF0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0078AE3A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0002393D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">005BC618</t>
-  </si>
-  <si>
-    <t xml:space="preserve">00309035</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0066421B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">000619DB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">001B5CCB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">00C5C934</t>
-  </si>
-  <si>
-    <t xml:space="preserve">00194E07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">001F8FEB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">01186F45</t>
-  </si>
-  <si>
-    <t xml:space="preserve">00B6389E</t>
-  </si>
-  <si>
-    <t xml:space="preserve">02F4ABBE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0089C876</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0204A7B9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">009EB58B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">00B7DBB2</t>
   </si>
 </sst>
 </file>
@@ -940,35 +820,35 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -976,19 +856,19 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -996,23 +876,23 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1020,15 +900,15 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1036,27 +916,27 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="14" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="14" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1069,47 +949,6 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="5">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD9D9D9"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF000000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFF66"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -1582,8 +1421,8 @@
         <f aca="false">IF(HEX2DEC(D21),HEX2DEC(D21)/HEX2DEC(E21),0)</f>
         <v>0</v>
       </c>
-      <c r="G21" s="21" t="s">
-        <v>32</v>
+      <c r="G21" s="21" t="n">
+        <v>343640</v>
       </c>
       <c r="H21" s="25" t="n">
         <f aca="false">IF(HEX2DEC(D21),HEX2DEC(G21)/HEX2DEC(D21),0.0001)</f>
@@ -1595,7 +1434,7 @@
         <v>2</v>
       </c>
       <c r="C22" s="19" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D22" s="24" t="s">
         <v>31</v>
@@ -1607,8 +1446,8 @@
         <f aca="false">IF(HEX2DEC(D22),HEX2DEC(D22)/HEX2DEC(E22),0)</f>
         <v>0</v>
       </c>
-      <c r="G22" s="21" t="s">
-        <v>34</v>
+      <c r="G22" s="21" t="n">
+        <v>1599254</v>
       </c>
       <c r="H22" s="25" t="n">
         <f aca="false">IF(HEX2DEC(D22),HEX2DEC(G22)/HEX2DEC(D22),0.0001)</f>
@@ -1620,7 +1459,7 @@
         <v>3</v>
       </c>
       <c r="C23" s="19" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D23" s="24" t="s">
         <v>31</v>
@@ -1632,8 +1471,8 @@
         <f aca="false">IF(HEX2DEC(D23),HEX2DEC(D23)/HEX2DEC(E23),0)</f>
         <v>0</v>
       </c>
-      <c r="G23" s="21" t="s">
-        <v>36</v>
+      <c r="G23" s="21" t="n">
+        <v>4130786</v>
       </c>
       <c r="H23" s="25" t="n">
         <f aca="false">IF(HEX2DEC(D23),HEX2DEC(G23)/HEX2DEC(D23),0.0001)</f>
@@ -1645,7 +1484,7 @@
         <v>4</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D24" s="24" t="s">
         <v>31</v>
@@ -1657,8 +1496,8 @@
         <f aca="false">IF(HEX2DEC(D24),HEX2DEC(D24)/HEX2DEC(E24),0)</f>
         <v>0</v>
       </c>
-      <c r="G24" s="21" t="s">
-        <v>38</v>
+      <c r="G24" s="21" t="n">
+        <v>2583293</v>
       </c>
       <c r="H24" s="25" t="n">
         <f aca="false">IF(HEX2DEC(D24),HEX2DEC(G24)/HEX2DEC(D24),0.0001)</f>
@@ -1670,7 +1509,7 @@
         <v>5</v>
       </c>
       <c r="C25" s="19" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D25" s="24" t="s">
         <v>31</v>
@@ -1682,8 +1521,8 @@
         <f aca="false">IF(HEX2DEC(D25),HEX2DEC(D25)/HEX2DEC(E25),0)</f>
         <v>0</v>
       </c>
-      <c r="G25" s="21" t="s">
-        <v>40</v>
+      <c r="G25" s="21" t="n">
+        <v>46601</v>
       </c>
       <c r="H25" s="25" t="n">
         <f aca="false">IF(HEX2DEC(D25),HEX2DEC(G25)/HEX2DEC(D25),0.0001)</f>
@@ -1695,7 +1534,7 @@
         <v>6</v>
       </c>
       <c r="C26" s="19" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="D26" s="24" t="s">
         <v>31</v>
@@ -1707,8 +1546,8 @@
         <f aca="false">IF(HEX2DEC(D26),HEX2DEC(D26)/HEX2DEC(E26),0)</f>
         <v>0</v>
       </c>
-      <c r="G26" s="21" t="s">
-        <v>42</v>
+      <c r="G26" s="21" t="n">
+        <v>1969534</v>
       </c>
       <c r="H26" s="25" t="n">
         <f aca="false">IF(HEX2DEC(D26),HEX2DEC(G26)/HEX2DEC(D26),0.0001)</f>
@@ -1720,7 +1559,7 @@
         <v>7</v>
       </c>
       <c r="C27" s="19" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="D27" s="24" t="s">
         <v>31</v>
@@ -1732,8 +1571,8 @@
         <f aca="false">IF(HEX2DEC(D27),HEX2DEC(D27)/HEX2DEC(E27),0)</f>
         <v>0</v>
       </c>
-      <c r="G27" s="21" t="s">
-        <v>44</v>
+      <c r="G27" s="21" t="n">
+        <v>1041006</v>
       </c>
       <c r="H27" s="25" t="n">
         <f aca="false">IF(HEX2DEC(D27),HEX2DEC(G27)/HEX2DEC(D27),0.0001)</f>
@@ -1745,7 +1584,7 @@
         <v>8</v>
       </c>
       <c r="C28" s="19" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="D28" s="24" t="s">
         <v>31</v>
@@ -1757,8 +1596,8 @@
         <f aca="false">IF(HEX2DEC(D28),HEX2DEC(D28)/HEX2DEC(E28),0)</f>
         <v>0</v>
       </c>
-      <c r="G28" s="21" t="s">
-        <v>46</v>
+      <c r="G28" s="21" t="n">
+        <v>2190475</v>
       </c>
       <c r="H28" s="25" t="n">
         <f aca="false">IF(HEX2DEC(D28),HEX2DEC(G28)/HEX2DEC(D28),0.0001)</f>
@@ -1770,7 +1609,7 @@
         <v>9</v>
       </c>
       <c r="C29" s="19" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="D29" s="24" t="s">
         <v>31</v>
@@ -1782,8 +1621,8 @@
         <f aca="false">IF(HEX2DEC(D29),HEX2DEC(D29)/HEX2DEC(E29),0)</f>
         <v>0</v>
       </c>
-      <c r="G29" s="21" t="s">
-        <v>48</v>
+      <c r="G29" s="21" t="n">
+        <v>130647</v>
       </c>
       <c r="H29" s="25" t="n">
         <f aca="false">IF(HEX2DEC(D29),HEX2DEC(G29)/HEX2DEC(D29),0.0001)</f>
@@ -1795,7 +1634,7 @@
         <v>10</v>
       </c>
       <c r="C30" s="19" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="D30" s="24" t="s">
         <v>31</v>
@@ -1807,8 +1646,8 @@
         <f aca="false">IF(HEX2DEC(D30),HEX2DEC(D30)/HEX2DEC(E30),0)</f>
         <v>0</v>
       </c>
-      <c r="G30" s="21" t="s">
-        <v>50</v>
+      <c r="G30" s="21" t="n">
+        <v>581771</v>
       </c>
       <c r="H30" s="25" t="n">
         <f aca="false">IF(HEX2DEC(D30),HEX2DEC(G30)/HEX2DEC(D30),0.0001)</f>
@@ -1820,7 +1659,7 @@
         <v>11</v>
       </c>
       <c r="C31" s="19" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="D31" s="24" t="s">
         <v>31</v>
@@ -1832,8 +1671,8 @@
         <f aca="false">IF(HEX2DEC(D31),HEX2DEC(D31)/HEX2DEC(E31),0)</f>
         <v>0</v>
       </c>
-      <c r="G31" s="21" t="s">
-        <v>52</v>
+      <c r="G31" s="21" t="n">
+        <v>4240749</v>
       </c>
       <c r="H31" s="25" t="n">
         <f aca="false">IF(HEX2DEC(D31),HEX2DEC(G31)/HEX2DEC(D31),0.0001)</f>
@@ -1845,7 +1684,7 @@
         <v>12</v>
       </c>
       <c r="C32" s="19" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="D32" s="24" t="s">
         <v>31</v>
@@ -1857,8 +1696,8 @@
         <f aca="false">IF(HEX2DEC(D32),HEX2DEC(D32)/HEX2DEC(E32),0)</f>
         <v>0</v>
       </c>
-      <c r="G32" s="21" t="s">
-        <v>54</v>
+      <c r="G32" s="21" t="n">
+        <v>545430</v>
       </c>
       <c r="H32" s="25" t="n">
         <f aca="false">IF(HEX2DEC(D32),HEX2DEC(G32)/HEX2DEC(D32),0.0001)</f>
@@ -1870,7 +1709,7 @@
         <v>13</v>
       </c>
       <c r="C33" s="19" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="D33" s="24" t="s">
         <v>31</v>
@@ -1882,8 +1721,8 @@
         <f aca="false">IF(HEX2DEC(D33),HEX2DEC(D33)/HEX2DEC(E33),0)</f>
         <v>0</v>
       </c>
-      <c r="G33" s="21" t="s">
-        <v>56</v>
+      <c r="G33" s="21" t="n">
+        <v>676520</v>
       </c>
       <c r="H33" s="25" t="n">
         <f aca="false">IF(HEX2DEC(D33),HEX2DEC(G33)/HEX2DEC(D33),0.0001)</f>
@@ -1895,7 +1734,7 @@
         <v>14</v>
       </c>
       <c r="C34" s="19" t="s">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="D34" s="24" t="s">
         <v>31</v>
@@ -1907,8 +1746,8 @@
         <f aca="false">IF(HEX2DEC(D34),HEX2DEC(D34)/HEX2DEC(E34),0)</f>
         <v>0</v>
       </c>
-      <c r="G34" s="21" t="s">
-        <v>58</v>
+      <c r="G34" s="21" t="n">
+        <v>6038605</v>
       </c>
       <c r="H34" s="25" t="n">
         <f aca="false">IF(HEX2DEC(D34),HEX2DEC(G34)/HEX2DEC(D34),0.0001)</f>
@@ -1920,7 +1759,7 @@
         <v>15</v>
       </c>
       <c r="C35" s="19" t="s">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="D35" s="24" t="s">
         <v>31</v>
@@ -1932,8 +1771,8 @@
         <f aca="false">IF(HEX2DEC(D35),HEX2DEC(D35)/HEX2DEC(E35),0)</f>
         <v>0</v>
       </c>
-      <c r="G35" s="21" t="s">
-        <v>60</v>
+      <c r="G35" s="21" t="n">
+        <v>3906531</v>
       </c>
       <c r="H35" s="25" t="n">
         <f aca="false">IF(HEX2DEC(D35),HEX2DEC(G35)/HEX2DEC(D35),0.0001)</f>
@@ -1945,7 +1784,7 @@
         <v>16</v>
       </c>
       <c r="C36" s="19" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="D36" s="24" t="s">
         <v>31</v>
@@ -1957,8 +1796,8 @@
         <f aca="false">IF(HEX2DEC(D36),HEX2DEC(D36)/HEX2DEC(E36),0)</f>
         <v>0</v>
       </c>
-      <c r="G36" s="21" t="s">
-        <v>62</v>
+      <c r="G36" s="21" t="n">
+        <v>16232737</v>
       </c>
       <c r="H36" s="25" t="n">
         <f aca="false">IF(HEX2DEC(D36),HEX2DEC(G36)/HEX2DEC(D36),0.0001)</f>
@@ -1970,7 +1809,7 @@
         <v>17</v>
       </c>
       <c r="C37" s="19" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="D37" s="24" t="s">
         <v>31</v>
@@ -1982,8 +1821,8 @@
         <f aca="false">IF(HEX2DEC(D37),HEX2DEC(D37)/HEX2DEC(E37),0)</f>
         <v>0</v>
       </c>
-      <c r="G37" s="21" t="s">
-        <v>64</v>
+      <c r="G37" s="21" t="n">
+        <v>2958023</v>
       </c>
       <c r="H37" s="25" t="n">
         <f aca="false">IF(HEX2DEC(D37),HEX2DEC(G37)/HEX2DEC(D37),0.0001)</f>
@@ -1995,7 +1834,7 @@
         <v>18</v>
       </c>
       <c r="C38" s="19" t="s">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="D38" s="24" t="s">
         <v>31</v>
@@ -2007,8 +1846,8 @@
         <f aca="false">IF(HEX2DEC(D38),HEX2DEC(D38)/HEX2DEC(E38),0)</f>
         <v>0</v>
       </c>
-      <c r="G38" s="21" t="s">
-        <v>66</v>
+      <c r="G38" s="21" t="n">
+        <v>11084756</v>
       </c>
       <c r="H38" s="25" t="n">
         <f aca="false">IF(HEX2DEC(D38),HEX2DEC(G38)/HEX2DEC(D38),0.0001)</f>
@@ -2020,7 +1859,7 @@
         <v>19</v>
       </c>
       <c r="C39" s="19" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="D39" s="24" t="s">
         <v>31</v>
@@ -2032,8 +1871,8 @@
         <f aca="false">IF(HEX2DEC(D39),HEX2DEC(D39)/HEX2DEC(E39),0)</f>
         <v>0</v>
       </c>
-      <c r="G39" s="21" t="s">
-        <v>68</v>
+      <c r="G39" s="21" t="n">
+        <v>3395161</v>
       </c>
       <c r="H39" s="25" t="n">
         <f aca="false">IF(HEX2DEC(D39),HEX2DEC(G39)/HEX2DEC(D39),0.0001)</f>
@@ -2045,7 +1884,7 @@
         <v>20</v>
       </c>
       <c r="C40" s="19" t="s">
-        <v>69</v>
+        <v>50</v>
       </c>
       <c r="D40" s="24" t="s">
         <v>31</v>
@@ -2057,8 +1896,8 @@
         <f aca="false">IF(HEX2DEC(D40),HEX2DEC(D40)/HEX2DEC(E40),0)</f>
         <v>0</v>
       </c>
-      <c r="G40" s="21" t="s">
-        <v>70</v>
+      <c r="G40" s="21" t="n">
+        <v>3942826</v>
       </c>
       <c r="H40" s="25" t="n">
         <f aca="false">IF(HEX2DEC(D40),HEX2DEC(G40)/HEX2DEC(D40),0.0001)</f>
@@ -2067,7 +1906,7 @@
     </row>
     <row r="42" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="8" t="s">
-        <v>71</v>
+        <v>51</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2075,12 +1914,12 @@
     </row>
     <row r="44" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B44" s="2" t="s">
-        <v>72</v>
+        <v>52</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" s="2"/>
       <c r="E44" s="26" t="s">
-        <v>73</v>
+        <v>53</v>
       </c>
       <c r="F44" s="26"/>
       <c r="G44" s="10"/>
@@ -2088,7 +1927,7 @@
     </row>
     <row r="45" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B45" s="27" t="s">
-        <v>74</v>
+        <v>54</v>
       </c>
       <c r="C45" s="27"/>
       <c r="D45" s="27"/>
@@ -2101,7 +1940,7 @@
     </row>
     <row r="46" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B46" s="27" t="s">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="C46" s="27"/>
       <c r="D46" s="27"/>
@@ -2112,7 +1951,7 @@
     </row>
     <row r="47" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B47" s="27" t="s">
-        <v>76</v>
+        <v>56</v>
       </c>
       <c r="C47" s="27"/>
       <c r="D47" s="27"/>
@@ -2123,7 +1962,7 @@
     </row>
     <row r="48" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B48" s="27" t="s">
-        <v>77</v>
+        <v>57</v>
       </c>
       <c r="C48" s="27"/>
       <c r="D48" s="27"/>
@@ -2134,7 +1973,7 @@
     </row>
     <row r="49" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B49" s="27" t="s">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="C49" s="27"/>
       <c r="D49" s="27"/>
@@ -2145,7 +1984,7 @@
     </row>
     <row r="50" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>79</v>
+        <v>59</v>
       </c>
       <c r="B50" s="10"/>
       <c r="C50" s="10"/>
@@ -2157,7 +1996,7 @@
     </row>
     <row r="51" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="29" t="s">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="B51" s="10"/>
       <c r="C51" s="10"/>
@@ -2169,7 +2008,7 @@
     </row>
     <row r="52" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="29" t="s">
-        <v>81</v>
+        <v>61</v>
       </c>
       <c r="B52" s="10"/>
       <c r="C52" s="10"/>
@@ -2181,7 +2020,7 @@
     </row>
     <row r="53" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
-        <v>82</v>
+        <v>62</v>
       </c>
       <c r="B53" s="10"/>
       <c r="C53" s="10"/>
@@ -2193,7 +2032,7 @@
     </row>
     <row r="54" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
-        <v>83</v>
+        <v>63</v>
       </c>
       <c r="B54" s="10"/>
       <c r="C54" s="10"/>
@@ -2205,7 +2044,7 @@
     </row>
     <row r="55" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
-        <v>84</v>
+        <v>64</v>
       </c>
       <c r="B55" s="10"/>
       <c r="C55" s="10"/>
@@ -2283,10 +2122,10 @@
   <dimension ref="A1:E23"/>
   <sheetFormatPr defaultColWidth="15.75" defaultRowHeight="30" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="5" width="9.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="5" width="14.51"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="30" width="22.25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="5" width="22.25"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2303,17 +2142,17 @@
         <v>22</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>85</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="18" t="s">
-        <v>86</v>
+        <v>66</v>
       </c>
       <c r="D2" s="18" t="s">
-        <v>87</v>
+        <v>67</v>
       </c>
       <c r="E2" s="2"/>
     </row>
@@ -2339,15 +2178,15 @@
       <c r="B4" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="C4" s="21" t="s">
-        <v>32</v>
-      </c>
-      <c r="D4" s="21" t="s">
-        <v>88</v>
+      <c r="C4" s="21" t="n">
+        <v>343640</v>
+      </c>
+      <c r="D4" s="21" t="n">
+        <v>1051297</v>
       </c>
       <c r="E4" s="22" t="n">
         <f aca="false">IF(HEX2DEC(C4),HEX2DEC(C4)/HEX2DEC(D4),0)</f>
-        <v>0.326860619759471</v>
+        <v>0.199990005643013</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2355,17 +2194,17 @@
         <v>2</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="C5" s="21" t="s">
-        <v>34</v>
-      </c>
-      <c r="D5" s="21" t="s">
-        <v>89</v>
+        <v>32</v>
+      </c>
+      <c r="C5" s="21" t="n">
+        <v>1599254</v>
+      </c>
+      <c r="D5" s="21" t="n">
+        <v>4888318</v>
       </c>
       <c r="E5" s="22" t="n">
         <f aca="false">IF(HEX2DEC(C5),HEX2DEC(C5)/HEX2DEC(D5),0)</f>
-        <v>0.327144629709051</v>
+        <v>0.297775093182173</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2373,17 +2212,17 @@
         <v>3</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>35</v>
-      </c>
-      <c r="C6" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="D6" s="21" t="s">
-        <v>90</v>
+        <v>33</v>
+      </c>
+      <c r="C6" s="21" t="n">
+        <v>4130786</v>
+      </c>
+      <c r="D6" s="21" t="n">
+        <v>12625378</v>
       </c>
       <c r="E6" s="22" t="n">
         <f aca="false">IF(HEX2DEC(C6),HEX2DEC(C6)/HEX2DEC(D6),0)</f>
-        <v>0.327185569769546</v>
+        <v>0.221622849201241</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2391,17 +2230,17 @@
         <v>4</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>37</v>
-      </c>
-      <c r="C7" s="21" t="s">
-        <v>38</v>
-      </c>
-      <c r="D7" s="21" t="s">
-        <v>91</v>
+        <v>34</v>
+      </c>
+      <c r="C7" s="21" t="n">
+        <v>2583293</v>
+      </c>
+      <c r="D7" s="21" t="n">
+        <v>7915229</v>
       </c>
       <c r="E7" s="22" t="n">
         <f aca="false">IF(HEX2DEC(C7),HEX2DEC(C7)/HEX2DEC(D7),0)</f>
-        <v>0.326597354228554</v>
+        <v>0.30980801566488</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2409,17 +2248,17 @@
         <v>5</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="C8" s="21" t="s">
-        <v>40</v>
-      </c>
-      <c r="D8" s="21" t="s">
-        <v>92</v>
+        <v>35</v>
+      </c>
+      <c r="C8" s="21" t="n">
+        <v>46601</v>
+      </c>
+      <c r="D8" s="21" t="n">
+        <v>144543</v>
       </c>
       <c r="E8" s="22" t="n">
         <f aca="false">IF(HEX2DEC(C8),HEX2DEC(C8)/HEX2DEC(D8),0)</f>
-        <v>0.322621375879225</v>
+        <v>0.216987303257704</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2427,17 +2266,17 @@
         <v>6</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>41</v>
-      </c>
-      <c r="C9" s="21" t="s">
-        <v>42</v>
-      </c>
-      <c r="D9" s="21" t="s">
-        <v>93</v>
+        <v>36</v>
+      </c>
+      <c r="C9" s="21" t="n">
+        <v>1969534</v>
+      </c>
+      <c r="D9" s="21" t="n">
+        <v>6021174</v>
       </c>
       <c r="E9" s="22" t="n">
         <f aca="false">IF(HEX2DEC(C9),HEX2DEC(C9)/HEX2DEC(D9),0)</f>
-        <v>0.327167333279242</v>
+        <v>0.264346425587692</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2445,17 +2284,17 @@
         <v>7</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>43</v>
-      </c>
-      <c r="C10" s="21" t="s">
-        <v>44</v>
-      </c>
-      <c r="D10" s="21" t="s">
-        <v>94</v>
+        <v>37</v>
+      </c>
+      <c r="C10" s="21" t="n">
+        <v>1041006</v>
+      </c>
+      <c r="D10" s="21" t="n">
+        <v>3182355</v>
       </c>
       <c r="E10" s="22" t="n">
         <f aca="false">IF(HEX2DEC(C10),HEX2DEC(C10)/HEX2DEC(D10),0)</f>
-        <v>0.327096173151577</v>
+        <v>0.328304646895993</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2463,17 +2302,17 @@
         <v>8</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>45</v>
-      </c>
-      <c r="C11" s="21" t="s">
-        <v>46</v>
-      </c>
-      <c r="D11" s="21" t="s">
-        <v>95</v>
+        <v>38</v>
+      </c>
+      <c r="C11" s="21" t="n">
+        <v>2190475</v>
+      </c>
+      <c r="D11" s="21" t="n">
+        <v>6720475</v>
       </c>
       <c r="E11" s="22" t="n">
         <f aca="false">IF(HEX2DEC(C11),HEX2DEC(C11)/HEX2DEC(D11),0)</f>
-        <v>0.326216370878873</v>
+        <v>0.325461662969809</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2481,17 +2320,17 @@
         <v>9</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="C12" s="21" t="s">
-        <v>48</v>
-      </c>
-      <c r="D12" s="21" t="s">
-        <v>96</v>
+        <v>39</v>
+      </c>
+      <c r="C12" s="21" t="n">
+        <v>130647</v>
+      </c>
+      <c r="D12" s="21" t="n">
+        <v>401411</v>
       </c>
       <c r="E12" s="22" t="n">
         <f aca="false">IF(HEX2DEC(C12),HEX2DEC(C12)/HEX2DEC(D12),0)</f>
-        <v>0.325511773606613</v>
+        <v>0.296894515246196</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2499,17 +2338,17 @@
         <v>10</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="C13" s="21" t="s">
-        <v>50</v>
-      </c>
-      <c r="D13" s="21" t="s">
-        <v>97</v>
+        <v>40</v>
+      </c>
+      <c r="C13" s="21" t="n">
+        <v>581771</v>
+      </c>
+      <c r="D13" s="21" t="n">
+        <v>1798925</v>
       </c>
       <c r="E13" s="22" t="n">
         <f aca="false">IF(HEX2DEC(C13),HEX2DEC(C13)/HEX2DEC(D13),0)</f>
-        <v>0.324415704202535</v>
+        <v>0.233333067929622</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2517,17 +2356,17 @@
         <v>11</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>51</v>
-      </c>
-      <c r="C14" s="21" t="s">
-        <v>52</v>
-      </c>
-      <c r="D14" s="21" t="s">
-        <v>98</v>
+        <v>41</v>
+      </c>
+      <c r="C14" s="21" t="n">
+        <v>4240749</v>
+      </c>
+      <c r="D14" s="21" t="n">
+        <v>12960010</v>
       </c>
       <c r="E14" s="22" t="n">
         <f aca="false">IF(HEX2DEC(C14),HEX2DEC(C14)/HEX2DEC(D14),0)</f>
-        <v>0.327218737704539</v>
+        <v>0.222788651376595</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2535,17 +2374,17 @@
         <v>12</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>53</v>
-      </c>
-      <c r="C15" s="21" t="s">
-        <v>54</v>
-      </c>
-      <c r="D15" s="21" t="s">
-        <v>99</v>
+        <v>42</v>
+      </c>
+      <c r="C15" s="21" t="n">
+        <v>545430</v>
+      </c>
+      <c r="D15" s="21" t="n">
+        <v>1668123</v>
       </c>
       <c r="E15" s="22" t="n">
         <f aca="false">IF(HEX2DEC(C15),HEX2DEC(C15)/HEX2DEC(D15),0)</f>
-        <v>0.326971885128514</v>
+        <v>0.235224024978648</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2553,17 +2392,17 @@
         <v>13</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="C16" s="21" t="s">
-        <v>56</v>
-      </c>
-      <c r="D16" s="21" t="s">
-        <v>100</v>
+        <v>43</v>
+      </c>
+      <c r="C16" s="21" t="n">
+        <v>676520</v>
+      </c>
+      <c r="D16" s="21" t="n">
+        <v>2069036</v>
       </c>
       <c r="E16" s="22" t="n">
         <f aca="false">IF(HEX2DEC(C16),HEX2DEC(C16)/HEX2DEC(D16),0)</f>
-        <v>0.326972398292642</v>
+        <v>0.19938745135071</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2571,17 +2410,17 @@
         <v>14</v>
       </c>
       <c r="B17" s="19" t="s">
-        <v>57</v>
-      </c>
-      <c r="C17" s="21" t="s">
-        <v>58</v>
-      </c>
-      <c r="D17" s="21" t="s">
-        <v>101</v>
+        <v>44</v>
+      </c>
+      <c r="C17" s="21" t="n">
+        <v>6038605</v>
+      </c>
+      <c r="D17" s="21" t="n">
+        <v>18453597</v>
       </c>
       <c r="E17" s="22" t="n">
         <f aca="false">IF(HEX2DEC(C17),HEX2DEC(C17)/HEX2DEC(D17),0)</f>
-        <v>0.327230716870441</v>
+        <v>0.247782334491855</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2589,17 +2428,17 @@
         <v>15</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>59</v>
-      </c>
-      <c r="C18" s="21" t="s">
-        <v>60</v>
-      </c>
-      <c r="D18" s="21" t="s">
-        <v>102</v>
+        <v>45</v>
+      </c>
+      <c r="C18" s="21" t="n">
+        <v>3906531</v>
+      </c>
+      <c r="D18" s="21" t="n">
+        <v>11938942</v>
       </c>
       <c r="E18" s="22" t="n">
         <f aca="false">IF(HEX2DEC(C18),HEX2DEC(C18)/HEX2DEC(D18),0)</f>
-        <v>0.3272180495704</v>
+        <v>0.202775407466757</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2607,17 +2446,17 @@
         <v>16</v>
       </c>
       <c r="B19" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="C19" s="21" t="s">
-        <v>62</v>
-      </c>
-      <c r="D19" s="21" t="s">
-        <v>103</v>
+        <v>46</v>
+      </c>
+      <c r="C19" s="21" t="n">
+        <v>16232737</v>
+      </c>
+      <c r="D19" s="21" t="n">
+        <v>49602569</v>
       </c>
       <c r="E19" s="22" t="n">
         <f aca="false">IF(HEX2DEC(C19),HEX2DEC(C19)/HEX2DEC(D19),0)</f>
-        <v>0.32725885657884</v>
+        <v>0.301698738006503</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2625,17 +2464,17 @@
         <v>17</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>63</v>
-      </c>
-      <c r="C20" s="21" t="s">
-        <v>64</v>
-      </c>
-      <c r="D20" s="21" t="s">
-        <v>104</v>
+        <v>47</v>
+      </c>
+      <c r="C20" s="21" t="n">
+        <v>2958023</v>
+      </c>
+      <c r="D20" s="21" t="n">
+        <v>9041960</v>
       </c>
       <c r="E20" s="22" t="n">
         <f aca="false">IF(HEX2DEC(C20),HEX2DEC(C20)/HEX2DEC(D20),0)</f>
-        <v>0.32714194745148</v>
+        <v>0.286599707964079</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2643,17 +2482,17 @@
         <v>18</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>65</v>
-      </c>
-      <c r="C21" s="21" t="s">
-        <v>66</v>
-      </c>
-      <c r="D21" s="21" t="s">
-        <v>105</v>
+        <v>48</v>
+      </c>
+      <c r="C21" s="21" t="n">
+        <v>11084756</v>
+      </c>
+      <c r="D21" s="21" t="n">
+        <v>33873009</v>
       </c>
       <c r="E21" s="22" t="n">
         <f aca="false">IF(HEX2DEC(C21),HEX2DEC(C21)/HEX2DEC(D21),0)</f>
-        <v>0.327254086613709</v>
+        <v>0.330544813392459</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2661,17 +2500,17 @@
         <v>19</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>67</v>
-      </c>
-      <c r="C22" s="21" t="s">
-        <v>68</v>
-      </c>
-      <c r="D22" s="21" t="s">
-        <v>106</v>
+        <v>49</v>
+      </c>
+      <c r="C22" s="21" t="n">
+        <v>3395161</v>
+      </c>
+      <c r="D22" s="21" t="n">
+        <v>10376199</v>
       </c>
       <c r="E22" s="22" t="n">
         <f aca="false">IF(HEX2DEC(C22),HEX2DEC(C22)/HEX2DEC(D22),0)</f>
-        <v>0.327213312588217</v>
+        <v>0.1988056115474</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2679,17 +2518,17 @@
         <v>20</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>69</v>
-      </c>
-      <c r="C23" s="21" t="s">
-        <v>70</v>
-      </c>
-      <c r="D23" s="21" t="s">
-        <v>107</v>
+        <v>50</v>
+      </c>
+      <c r="C23" s="21" t="n">
+        <v>3942826</v>
+      </c>
+      <c r="D23" s="21" t="n">
+        <v>12050280</v>
       </c>
       <c r="E23" s="22" t="n">
         <f aca="false">IF(HEX2DEC(C23),HEX2DEC(C23)/HEX2DEC(D23),0)</f>
-        <v>0.327197030872256</v>
+        <v>0.198602837709332</v>
       </c>
     </row>
   </sheetData>

</xml_diff>